<commit_message>
Update Feature: Series Search 1.0
</commit_message>
<xml_diff>
--- a/excel_data/gcg_cardlist_limited.xlsx
+++ b/excel_data/gcg_cardlist_limited.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FLC\Desktop\JavaScript\Gundam Card Web\gundam-card-web\excel_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA9D916C-F97B-488C-ACE8-71F3A5F201CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A796D7ED-1E01-4254-8DE4-8C54034E8443}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2220" yWindow="4090" windowWidth="21780" windowHeight="16940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1210" yWindow="2920" windowWidth="20380" windowHeight="16940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="限定商品_Data" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="137">
   <si>
     <t>序號</t>
   </si>
@@ -440,6 +440,29 @@
   <si>
     <t>豪華卡牌收藏 拼裝鋼彈套裝 -機動戰士Gundam GQuuuuuuX- [PC02A]</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>出自作品</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>機動戦士ガンダム</t>
+  </si>
+  <si>
+    <t>新機動戦記ガンダムW</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>機動戦士ガンダム 鉄血のオルフェンズ</t>
+  </si>
+  <si>
+    <t>機動戦士Gundam GQuuuuuuX(ジークアクス)</t>
+  </si>
+  <si>
+    <t>機動戦士ガンダムSEED</t>
+  </si>
+  <si>
+    <t>機動戦士ガンダム 水星の魔女</t>
   </si>
 </sst>
 </file>
@@ -793,14 +816,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="3" width="14" customWidth="1"/>
-    <col min="4" max="5" width="70.09765625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="32.3984375" customWidth="1"/>
+    <col min="5" max="5" width="34.5" customWidth="1"/>
+    <col min="6" max="6" width="40.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -816,8 +841,11 @@
       <c r="E1" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -833,8 +861,11 @@
       <c r="E2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F2" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -850,8 +881,11 @@
       <c r="E3" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F3" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -867,8 +901,11 @@
       <c r="E4" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -884,8 +921,11 @@
       <c r="E5" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F5" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -901,8 +941,11 @@
       <c r="E6" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F6" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -918,8 +961,11 @@
       <c r="E7" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F7" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -935,8 +981,11 @@
       <c r="E8" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F8" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -952,8 +1001,11 @@
       <c r="E9" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F9" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>27</v>
       </c>
@@ -969,8 +1021,11 @@
       <c r="E10" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F10" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>29</v>
       </c>
@@ -986,8 +1041,11 @@
       <c r="E11" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F11" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>31</v>
       </c>
@@ -1003,8 +1061,11 @@
       <c r="E12" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F12" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>34</v>
       </c>
@@ -1020,8 +1081,11 @@
       <c r="E13" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F13" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>36</v>
       </c>
@@ -1037,8 +1101,11 @@
       <c r="E14" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F14" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>39</v>
       </c>
@@ -1054,8 +1121,11 @@
       <c r="E15" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F15" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>42</v>
       </c>
@@ -1071,8 +1141,11 @@
       <c r="E16" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F16" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>44</v>
       </c>
@@ -1088,8 +1161,11 @@
       <c r="E17" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F17" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>47</v>
       </c>
@@ -1105,8 +1181,11 @@
       <c r="E18" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F18" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>49</v>
       </c>
@@ -1122,8 +1201,11 @@
       <c r="E19" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F19" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>51</v>
       </c>
@@ -1139,8 +1221,11 @@
       <c r="E20" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F20" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>53</v>
       </c>
@@ -1156,8 +1241,11 @@
       <c r="E21" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F21" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>55</v>
       </c>
@@ -1173,8 +1261,11 @@
       <c r="E22" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F22" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>57</v>
       </c>
@@ -1190,8 +1281,11 @@
       <c r="E23" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F23" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>59</v>
       </c>
@@ -1207,8 +1301,11 @@
       <c r="E24" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F24" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>61</v>
       </c>
@@ -1224,8 +1321,11 @@
       <c r="E25" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F25" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>63</v>
       </c>
@@ -1241,8 +1341,11 @@
       <c r="E26" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F26" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>66</v>
       </c>
@@ -1258,8 +1361,11 @@
       <c r="E27" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F27" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>68</v>
       </c>
@@ -1275,8 +1381,11 @@
       <c r="E28" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F28" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>70</v>
       </c>
@@ -1292,8 +1401,11 @@
       <c r="E29" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F29" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>72</v>
       </c>
@@ -1309,8 +1421,11 @@
       <c r="E30" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F30" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>74</v>
       </c>
@@ -1326,8 +1441,11 @@
       <c r="E31" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F31" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>76</v>
       </c>
@@ -1343,8 +1461,11 @@
       <c r="E32" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F32" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>78</v>
       </c>
@@ -1360,8 +1481,11 @@
       <c r="E33" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F33" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>80</v>
       </c>
@@ -1377,8 +1501,11 @@
       <c r="E34" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F34" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>82</v>
       </c>
@@ -1394,8 +1521,11 @@
       <c r="E35" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F35" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>84</v>
       </c>
@@ -1411,8 +1541,11 @@
       <c r="E36" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F36" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>86</v>
       </c>
@@ -1428,8 +1561,11 @@
       <c r="E37" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F37" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>88</v>
       </c>
@@ -1445,8 +1581,11 @@
       <c r="E38" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F38" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>90</v>
       </c>
@@ -1462,8 +1601,11 @@
       <c r="E39" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F39" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>92</v>
       </c>
@@ -1479,8 +1621,11 @@
       <c r="E40" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F40" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>94</v>
       </c>
@@ -1496,8 +1641,11 @@
       <c r="E41" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F41" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>96</v>
       </c>
@@ -1513,8 +1661,11 @@
       <c r="E42" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F42" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>98</v>
       </c>
@@ -1530,8 +1681,11 @@
       <c r="E43" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F43" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>100</v>
       </c>
@@ -1547,8 +1701,11 @@
       <c r="E44" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F44" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>102</v>
       </c>
@@ -1564,8 +1721,11 @@
       <c r="E45" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F45" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>104</v>
       </c>
@@ -1581,8 +1741,11 @@
       <c r="E46" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F46" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>106</v>
       </c>
@@ -1598,8 +1761,11 @@
       <c r="E47" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F47" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>108</v>
       </c>
@@ -1615,8 +1781,11 @@
       <c r="E48" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F48" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>110</v>
       </c>
@@ -1632,8 +1801,11 @@
       <c r="E49" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F49" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>112</v>
       </c>
@@ -1649,8 +1821,11 @@
       <c r="E50" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F50" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>114</v>
       </c>
@@ -1666,8 +1841,11 @@
       <c r="E51" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F51" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>116</v>
       </c>
@@ -1683,8 +1861,11 @@
       <c r="E52" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F52" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>118</v>
       </c>
@@ -1700,8 +1881,11 @@
       <c r="E53" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F53" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>120</v>
       </c>
@@ -1717,8 +1901,11 @@
       <c r="E54" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F54" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>122</v>
       </c>
@@ -1733,6 +1920,9 @@
       </c>
       <c r="E55" t="s">
         <v>129</v>
+      </c>
+      <c r="F55" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>